<commit_message>
Dashboard 2026-08-28 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339349971/spec-339349971.xlsx
+++ b/vse-loti/339349971/spec-339349971.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.00&quot; ₽&quot;"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00&quot; ₽&quot;"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -60,13 +61,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -500,27 +504,210 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Труба стальная горячекатаная Ф-57х4 ГОСТ 8732-78 (марка стали Ст.20)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>293466.6</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Труба стальная горячекатаная Ф-76х4 ГОСТ 8732-78 (марка стали Ст.20)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Труба стальная горячекатаная Ф-89х5 ГОСТ 8732-78 (марка стали Ст.20)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>293466.6</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Труба стальная горячекатаная Ф-108х5 ГОСТ 8732-78 (марка стали Ст.20)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>293466.6</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Труба стальная горячекатаная Ф-219х6 ГОСТ 8732-78 (марка стали Ст.20)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>т</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>440199.9</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>146733.3</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>176079.96</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="H2" s="3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="E7" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>1467333</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>НМЦК из обоснования:</t>
         </is>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="H8" s="6" t="n">
         <v>1467333</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Источник: 852308699.txt</t>
         </is>

</xml_diff>